<commit_message>
add stock frontend, changed item import logic
</commit_message>
<xml_diff>
--- a/test_file/test_stocks.xlsx
+++ b/test_file/test_stocks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Rolan\ProgProjs\digital_inventory_system\test_file\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26156850-22F4-44F3-8D67-99B2483E0FB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96F17209-9617-4A08-99A6-54135C4CAE72}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{80F44311-33CB-4E50-B7EB-75652C6FECB9}"/>
   </bookViews>
@@ -45,9 +45,6 @@
     <t>condition</t>
   </si>
   <si>
-    <t>AAA</t>
-  </si>
-  <si>
     <t>available</t>
   </si>
   <si>
@@ -57,10 +54,13 @@
     <t>Working</t>
   </si>
   <si>
-    <t>AAAbbb</t>
-  </si>
-  <si>
     <t>borrowed</t>
+  </si>
+  <si>
+    <t>AAAbbba</t>
+  </si>
+  <si>
+    <t>AAAa</t>
   </si>
 </sst>
 </file>
@@ -433,13 +433,13 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B2" t="s">
         <v>3</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>4</v>
-      </c>
-      <c r="C2" t="s">
-        <v>5</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
@@ -447,10 +447,10 @@
         <v>7</v>
       </c>
       <c r="B3" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>